<commit_message>
Atualiza dashboard 24/08/2026 17:08:03,42
</commit_message>
<xml_diff>
--- a/Escala_2026.xlsx
+++ b/Escala_2026.xlsx
@@ -60,7 +60,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -116,6 +116,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE5CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -279,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -374,6 +379,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2315,14 +2323,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="DC2" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DD2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DC2" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="DD2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DE2" s="32" t="inlineStr">
@@ -2335,9 +2343,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DG2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DG2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DH2" s="28" t="inlineStr">
@@ -2350,14 +2358,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="DJ2" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DK2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DJ2" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="DK2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DL2" s="32" t="inlineStr">
@@ -2365,9 +2373,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DM2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DM2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DN2" s="32" t="inlineStr">
@@ -2385,9 +2393,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="DQ2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DQ2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DR2" s="32" t="inlineStr">
@@ -2395,14 +2403,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DS2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DT2" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="DS2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="DT2" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="DU2" s="32" t="inlineStr">
@@ -2425,19 +2433,19 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DY2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DZ2" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="EA2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DY2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="DZ2" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="EA2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EB2" s="32" t="inlineStr">
@@ -2455,19 +2463,19 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="EE2" s="26" t="inlineStr">
+      <c r="EE2" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
       </c>
-      <c r="EF2" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="EG2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EF2" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="EG2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EH2" s="32" t="inlineStr">
@@ -2475,9 +2483,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EI2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EI2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EJ2" s="28" t="inlineStr">
@@ -2495,9 +2503,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EM2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EM2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EN2" s="32" t="inlineStr">
@@ -2540,9 +2548,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EV2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EV2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EW2" s="32" t="inlineStr">
@@ -2560,19 +2568,19 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="EZ2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FA2" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FB2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EZ2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="FA2" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="FB2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FC2" s="32" t="inlineStr">
@@ -2595,9 +2603,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="FG2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FG2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FH2" s="32" t="inlineStr">
@@ -2630,7 +2638,7 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="FN2" s="26" t="inlineStr">
+      <c r="FN2" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -2640,9 +2648,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FP2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FP2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FQ2" s="32" t="inlineStr">
@@ -2670,9 +2678,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FV2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FV2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FW2" s="32" t="inlineStr">
@@ -2705,9 +2713,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GC2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GC2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GD2" s="32" t="inlineStr">
@@ -2735,7 +2743,7 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="GI2" s="26" t="inlineStr">
+      <c r="GI2" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -2745,9 +2753,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GK2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GK2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GL2" s="32" t="inlineStr">
@@ -2755,9 +2763,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GM2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GM2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GN2" s="28" t="inlineStr">
@@ -2810,22 +2818,22 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GX2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GY2" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="GZ2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HA2" s="26" t="inlineStr">
+      <c r="GX2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="GY2" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="GZ2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="HA2" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -2845,19 +2853,19 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HE2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HF2" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HG2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HE2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="HF2" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="HG2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HH2" s="32" t="inlineStr">
@@ -2885,9 +2893,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HM2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HM2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HN2" s="32" t="inlineStr">
@@ -2910,9 +2918,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="HR2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HR2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HS2" s="32" t="inlineStr">
@@ -2925,14 +2933,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HU2" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HV2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HU2" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="HV2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HW2" s="28" t="inlineStr">
@@ -2945,14 +2953,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="HY2" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HZ2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HY2" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="HZ2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IA2" s="32" t="inlineStr">
@@ -2960,9 +2968,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IB2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IB2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IC2" s="32" t="inlineStr">
@@ -2980,9 +2988,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="IF2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IF2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IG2" s="32" t="inlineStr">
@@ -2990,17 +2998,17 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IH2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="II2" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="IJ2" s="26" t="inlineStr">
+      <c r="IH2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="II2" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="IJ2" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -3030,9 +3038,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IP2" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IP2" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
     </row>
@@ -3572,19 +3580,19 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DD3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DE3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DF3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DD3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="DE3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="DF3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DG3" s="32" t="inlineStr">
@@ -3607,9 +3615,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DK3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DK3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DL3" s="32" t="inlineStr">
@@ -3642,19 +3650,19 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DR3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DS3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DT3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DR3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="DS3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="DT3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DU3" s="32" t="inlineStr">
@@ -3672,9 +3680,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="DX3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DX3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DY3" s="32" t="inlineStr">
@@ -3687,14 +3695,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EA3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="EB3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EA3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="EB3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EC3" s="28" t="inlineStr">
@@ -3707,24 +3715,24 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="EE3" s="26" t="inlineStr">
+      <c r="EE3" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
       </c>
-      <c r="EF3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EG3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="EH3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EF3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="EG3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="EH3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EI3" s="32" t="inlineStr">
@@ -3747,9 +3755,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EM3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EM3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EN3" s="32" t="inlineStr">
@@ -3777,9 +3785,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="ES3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="ES3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="ET3" s="32" t="inlineStr">
@@ -3787,9 +3795,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EU3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EU3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EV3" s="32" t="inlineStr">
@@ -3797,9 +3805,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EW3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="EW3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="EX3" s="28" t="inlineStr">
@@ -3812,9 +3820,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="EZ3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EZ3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FA3" s="32" t="inlineStr">
@@ -3827,14 +3835,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FC3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FD3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FC3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="FD3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FE3" s="28" t="inlineStr">
@@ -3862,9 +3870,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FJ3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FJ3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FK3" s="32" t="inlineStr">
@@ -3882,19 +3890,19 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="FN3" s="26" t="inlineStr">
+      <c r="FN3" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
       </c>
-      <c r="FO3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FP3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FO3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="FP3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FQ3" s="32" t="inlineStr">
@@ -3902,9 +3910,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FR3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FR3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FS3" s="28" t="inlineStr">
@@ -3922,9 +3930,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FV3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FV3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FW3" s="32" t="inlineStr">
@@ -3957,9 +3965,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GC3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GC3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GD3" s="32" t="inlineStr">
@@ -3987,7 +3995,7 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="GI3" s="26" t="inlineStr">
+      <c r="GI3" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -4002,9 +4010,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GL3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GL3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GM3" s="32" t="inlineStr">
@@ -4022,19 +4030,19 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="GP3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GQ3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="GR3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GP3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="GQ3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="GR3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GS3" s="32" t="inlineStr">
@@ -4067,9 +4075,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GY3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GY3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GZ3" s="32" t="inlineStr">
@@ -4077,7 +4085,7 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HA3" s="26" t="inlineStr">
+      <c r="HA3" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -4092,14 +4100,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="HD3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HE3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HD3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="HE3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HF3" s="32" t="inlineStr">
@@ -4107,9 +4115,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HG3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HG3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HH3" s="32" t="inlineStr">
@@ -4132,19 +4140,19 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HL3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HM3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HN3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HL3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="HM3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="HN3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HO3" s="32" t="inlineStr">
@@ -4167,9 +4175,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HS3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HS3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HT3" s="32" t="inlineStr">
@@ -4177,14 +4185,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HU3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HV3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="HU3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="HV3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="HW3" s="28" t="inlineStr">
@@ -4197,19 +4205,19 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="HY3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HZ3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="IA3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HY3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="HZ3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="IA3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IB3" s="32" t="inlineStr">
@@ -4232,14 +4240,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="IF3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="IG3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IF3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="IG3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IH3" s="32" t="inlineStr">
@@ -4247,12 +4255,12 @@
           <t>site</t>
         </is>
       </c>
-      <c r="II3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="IJ3" s="26" t="inlineStr">
+      <c r="II3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="IJ3" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -4267,9 +4275,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="IM3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IM3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IN3" s="32" t="inlineStr">
@@ -4277,14 +4285,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IO3" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="IP3" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="IO3" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="IP3" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
     </row>
@@ -4819,9 +4827,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="DC4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DC4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DD4" s="32" t="inlineStr">
@@ -4829,14 +4837,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DE4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DF4" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="DE4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="DF4" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="DG4" s="32" t="inlineStr">
@@ -4854,9 +4862,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="DJ4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DJ4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DK4" s="32" t="inlineStr">
@@ -4889,14 +4897,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="DQ4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DR4" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="DQ4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="DR4" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="DS4" s="32" t="inlineStr">
@@ -4904,9 +4912,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DT4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DT4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DU4" s="32" t="inlineStr">
@@ -4924,9 +4932,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="DX4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DX4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DY4" s="32" t="inlineStr">
@@ -4934,9 +4942,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DZ4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DZ4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EA4" s="32" t="inlineStr">
@@ -4944,9 +4952,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EB4" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="EB4" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="EC4" s="28" t="inlineStr">
@@ -4959,14 +4967,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="EE4" s="26" t="inlineStr">
+      <c r="EE4" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
       </c>
-      <c r="EF4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EF4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EG4" s="32" t="inlineStr">
@@ -5004,9 +5012,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EN4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EN4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EO4" s="32" t="inlineStr">
@@ -5029,9 +5037,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="ES4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="ES4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="ET4" s="32" t="inlineStr">
@@ -5064,14 +5072,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="EZ4" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FA4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EZ4" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="FA4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FB4" s="32" t="inlineStr">
@@ -5079,9 +5087,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FC4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FC4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FD4" s="32" t="inlineStr">
@@ -5104,9 +5112,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FH4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FH4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FI4" s="32" t="inlineStr">
@@ -5134,24 +5142,24 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="FN4" s="26" t="inlineStr">
+      <c r="FN4" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
       </c>
-      <c r="FO4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FP4" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FQ4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FO4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="FP4" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="FQ4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FR4" s="32" t="inlineStr">
@@ -5169,19 +5177,19 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="FU4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FV4" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FW4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FU4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="FV4" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="FW4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FX4" s="32" t="inlineStr">
@@ -5214,9 +5222,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GD4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GD4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GE4" s="32" t="inlineStr">
@@ -5239,7 +5247,7 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="GI4" s="26" t="inlineStr">
+      <c r="GI4" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -5249,19 +5257,19 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GK4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GL4" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="GM4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GK4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="GL4" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="GM4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GN4" s="28" t="inlineStr">
@@ -5294,9 +5302,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GT4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GT4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GU4" s="28" t="inlineStr">
@@ -5324,12 +5332,12 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GZ4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HA4" s="26" t="inlineStr">
+      <c r="GZ4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="HA4" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -5344,9 +5352,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="HD4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HD4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HE4" s="32" t="inlineStr">
@@ -5354,14 +5362,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HF4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HG4" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="HF4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="HG4" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="HH4" s="32" t="inlineStr">
@@ -5379,19 +5387,19 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="HK4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HL4" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HM4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HK4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="HL4" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="HM4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HN4" s="32" t="inlineStr">
@@ -5424,9 +5432,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HT4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HT4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HU4" s="32" t="inlineStr">
@@ -5449,9 +5457,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="HY4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HY4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HZ4" s="32" t="inlineStr">
@@ -5464,14 +5472,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IB4" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="IC4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IB4" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="IC4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="ID4" s="28" t="inlineStr">
@@ -5499,12 +5507,12 @@
           <t>site</t>
         </is>
       </c>
-      <c r="II4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="IJ4" s="26" t="inlineStr">
+      <c r="II4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="IJ4" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -5519,9 +5527,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="IM4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IM4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IN4" s="32" t="inlineStr">
@@ -5529,9 +5537,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IO4" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IO4" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IP4" s="32" t="inlineStr">
@@ -6071,9 +6079,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="DC5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DC5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DD5" s="32" t="inlineStr">
@@ -6111,14 +6119,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DK5" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DL5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DK5" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="DL5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DM5" s="32" t="inlineStr">
@@ -6126,9 +6134,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DN5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DN5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DO5" s="28" t="inlineStr">
@@ -6141,14 +6149,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="DQ5" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DR5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DQ5" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="DR5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DS5" s="32" t="inlineStr">
@@ -6161,9 +6169,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DU5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DU5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DV5" s="28" t="inlineStr">
@@ -6176,14 +6184,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="DX5" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DY5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DX5" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="DY5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DZ5" s="32" t="inlineStr">
@@ -6191,9 +6199,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EA5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EA5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EB5" s="32" t="inlineStr">
@@ -6211,7 +6219,7 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="EE5" s="26" t="inlineStr">
+      <c r="EE5" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -6221,9 +6229,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EG5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EG5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EH5" s="32" t="inlineStr">
@@ -6231,9 +6239,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EI5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EI5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EJ5" s="28" t="inlineStr">
@@ -6266,9 +6274,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EP5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EP5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EQ5" s="28" t="inlineStr">
@@ -6286,9 +6294,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="ET5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="ET5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EU5" s="32" t="inlineStr">
@@ -6296,14 +6304,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EV5" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="EW5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EV5" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="EW5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EX5" s="28" t="inlineStr">
@@ -6321,19 +6329,19 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FA5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FB5" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FC5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FA5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="FB5" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="FC5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FD5" s="32" t="inlineStr">
@@ -6371,9 +6379,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FK5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FK5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FL5" s="28" t="inlineStr">
@@ -6386,14 +6394,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="FN5" s="26" t="inlineStr">
+      <c r="FN5" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
       </c>
-      <c r="FO5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FO5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FP5" s="32" t="inlineStr">
@@ -6421,9 +6429,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="FU5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FU5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FV5" s="32" t="inlineStr">
@@ -6456,9 +6464,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="GB5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GB5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GC5" s="32" t="inlineStr">
@@ -6491,24 +6499,24 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="GI5" s="26" t="inlineStr">
+      <c r="GI5" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
       </c>
-      <c r="GJ5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GK5" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="GL5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GJ5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="GK5" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="GL5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GM5" s="32" t="inlineStr">
@@ -6526,14 +6534,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="GP5" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="GQ5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GP5" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="GQ5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GR5" s="32" t="inlineStr">
@@ -6541,9 +6549,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GS5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GS5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GT5" s="32" t="inlineStr">
@@ -6561,9 +6569,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="GW5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GW5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GX5" s="32" t="inlineStr">
@@ -6571,9 +6579,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GY5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GY5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GZ5" s="32" t="inlineStr">
@@ -6581,7 +6589,7 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HA5" s="26" t="inlineStr">
+      <c r="HA5" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -6596,14 +6604,14 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="HD5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HE5" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="HD5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="HE5" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="HF5" s="32" t="inlineStr">
@@ -6616,9 +6624,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HH5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HH5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HI5" s="28" t="inlineStr">
@@ -6636,9 +6644,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HL5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HL5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HM5" s="32" t="inlineStr">
@@ -6681,9 +6689,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HU5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HU5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HV5" s="32" t="inlineStr">
@@ -6706,19 +6714,19 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HZ5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="IA5" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="IB5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HZ5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="IA5" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="IB5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IC5" s="32" t="inlineStr">
@@ -6736,9 +6744,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="IF5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IF5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IG5" s="32" t="inlineStr">
@@ -6746,9 +6754,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IH5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IH5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="II5" s="32" t="inlineStr">
@@ -6756,7 +6764,7 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IJ5" s="26" t="inlineStr">
+      <c r="IJ5" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -6776,19 +6784,19 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IN5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="IO5" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="IP5" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IN5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="IO5" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="IP5" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
     </row>
@@ -7328,9 +7336,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DD6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="DD6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="DE6" s="32" t="inlineStr">
@@ -7343,9 +7351,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DG6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DG6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DH6" s="28" t="inlineStr">
@@ -7363,19 +7371,19 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DK6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DL6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DM6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="DK6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="DL6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="DM6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="DN6" s="32" t="inlineStr">
@@ -7408,14 +7416,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="DT6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DU6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="DT6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="DU6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="DV6" s="28" t="inlineStr">
@@ -7448,9 +7456,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EB6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EB6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EC6" s="28" t="inlineStr">
@@ -7463,7 +7471,7 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="EE6" s="26" t="inlineStr">
+      <c r="EE6" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -7478,14 +7486,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EH6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EI6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="EH6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="EI6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="EJ6" s="28" t="inlineStr">
@@ -7503,14 +7511,14 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EM6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="EN6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EM6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="EN6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EO6" s="32" t="inlineStr">
@@ -7518,9 +7526,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EP6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EP6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EQ6" s="28" t="inlineStr">
@@ -7533,9 +7541,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="ES6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="ES6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="ET6" s="32" t="inlineStr">
@@ -7553,9 +7561,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="EW6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="EW6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="EX6" s="28" t="inlineStr">
@@ -7578,9 +7586,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FB6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FB6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FC6" s="32" t="inlineStr">
@@ -7608,9 +7616,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FH6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FH6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FI6" s="32" t="inlineStr">
@@ -7623,9 +7631,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FK6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="FK6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="FL6" s="28" t="inlineStr">
@@ -7638,7 +7646,7 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="FN6" s="26" t="inlineStr">
+      <c r="FN6" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -7648,9 +7656,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FP6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FP6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FQ6" s="32" t="inlineStr">
@@ -7658,9 +7666,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FR6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FR6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FS6" s="28" t="inlineStr">
@@ -7673,9 +7681,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="FU6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="FU6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="FV6" s="32" t="inlineStr">
@@ -7688,9 +7696,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="FX6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="FX6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="FY6" s="32" t="inlineStr">
@@ -7728,9 +7736,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GF6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GF6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GG6" s="28" t="inlineStr">
@@ -7743,7 +7751,7 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="GI6" s="26" t="inlineStr">
+      <c r="GI6" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -7753,9 +7761,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GK6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GK6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GL6" s="32" t="inlineStr">
@@ -7763,9 +7771,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GM6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="GM6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="GN6" s="28" t="inlineStr">
@@ -7783,9 +7791,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GQ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GQ6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GR6" s="32" t="inlineStr">
@@ -7813,9 +7821,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="GW6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="GW6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="GX6" s="32" t="inlineStr">
@@ -7828,12 +7836,12 @@
           <t>site</t>
         </is>
       </c>
-      <c r="GZ6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HA6" s="26" t="inlineStr">
+      <c r="GZ6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="HA6" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -7848,9 +7856,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="HD6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HD6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HE6" s="32" t="inlineStr">
@@ -7858,9 +7866,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HF6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HF6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HG6" s="32" t="inlineStr">
@@ -7868,9 +7876,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="HH6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="HH6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="HI6" s="28" t="inlineStr">
@@ -7918,9 +7926,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="HR6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="HR6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="HS6" s="32" t="inlineStr">
@@ -7963,9 +7971,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IA6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IA6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IB6" s="32" t="inlineStr">
@@ -7973,9 +7981,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IC6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="IC6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="ID6" s="28" t="inlineStr">
@@ -7988,9 +7996,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="IF6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IF6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IG6" s="32" t="inlineStr">
@@ -7998,17 +8006,17 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IH6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="II6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="IJ6" s="26" t="inlineStr">
+      <c r="IH6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="II6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="IJ6" s="34" t="inlineStr">
         <is>
           <t>feriado</t>
         </is>
@@ -8023,9 +8031,9 @@
           <t>fds</t>
         </is>
       </c>
-      <c r="IM6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
+      <c r="IM6" s="32" t="inlineStr">
+        <is>
+          <t>site</t>
         </is>
       </c>
       <c r="IN6" s="32" t="inlineStr">
@@ -8033,9 +8041,9 @@
           <t>site</t>
         </is>
       </c>
-      <c r="IO6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
+      <c r="IO6" s="31" t="inlineStr">
+        <is>
+          <t>home</t>
         </is>
       </c>
       <c r="IP6" s="32" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboard 24/08/2026 17:12:18,54
</commit_message>
<xml_diff>
--- a/Escala_2026.xlsx
+++ b/Escala_2026.xlsx
@@ -482,16 +482,6 @@
         <t>Folga Banco de Horas</t>
       </text>
     </comment>
-    <comment ref="P6" authorId="0" shapeId="0">
-      <text>
-        <t>Folga banco de horas</t>
-      </text>
-    </comment>
-    <comment ref="W6" authorId="0" shapeId="0">
-      <text>
-        <t>Folga banco de Horas</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
@@ -817,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:IP6"/>
+  <dimension ref="A1:IP5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6800,1258 +6790,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>Samuel</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="E6" s="19" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="F6" s="20" t="inlineStr">
-        <is>
-          <t>feriado</t>
-        </is>
-      </c>
-      <c r="G6" s="21" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="I6" s="23" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="K6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="L6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="M6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="N6" s="21" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="O6" s="22" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="P6" s="17" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="Q6" s="19" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="R6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="S6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="T6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="U6" s="21" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="V6" s="22" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="W6" s="17" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="X6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="Y6" s="19" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="Z6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AA6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AB6" s="21" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="AC6" s="22" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="AD6" s="17" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AE6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AF6" s="19" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="AG6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AH6" s="18" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AI6" s="21" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="AJ6" s="22" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="AK6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AL6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AM6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="AN6" s="26" t="inlineStr">
-        <is>
-          <t>feriado</t>
-        </is>
-      </c>
-      <c r="AO6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AP6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="AQ6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="AR6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="AS6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AT6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AU6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AV6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AW6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="AX6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="AY6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="AZ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="BA6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="BB6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="BC6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="BD6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="BE6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="BF6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="BG6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="BH6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="BI6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="BJ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="BK6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="BL6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="BM6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="BN6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="BO6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="BP6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="BQ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="BR6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="BS6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="BT6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="BU6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="BV6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="BW6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="BX6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="BY6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="BZ6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="CA6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CB6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CC6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CD6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CE6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CF6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="CG6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="CH6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CI6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CJ6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CK6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CL6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CM6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="CN6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="CO6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CP6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CQ6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CR6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CS6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CT6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="CU6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="CV6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CW6" s="33" t="inlineStr">
-        <is>
-          <t>férias</t>
-        </is>
-      </c>
-      <c r="CX6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="CY6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="CZ6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DA6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="DB6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="DC6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DD6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DE6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DF6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DG6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DH6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="DI6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="DJ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DK6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DL6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DM6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DN6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DO6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="DP6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="DQ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DR6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DS6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DT6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DU6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DV6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="DW6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="DX6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="DY6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="DZ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EA6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EB6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="EC6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="ED6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="EE6" s="34" t="inlineStr">
-        <is>
-          <t>feriado</t>
-        </is>
-      </c>
-      <c r="EF6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EG6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EH6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="EI6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EJ6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="EK6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="EL6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EM6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EN6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="EO6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EP6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="EQ6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="ER6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="ES6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="ET6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EU6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EV6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="EW6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="EX6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="EY6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="EZ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FA6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FB6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FC6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FD6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FE6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="FF6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="FG6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FH6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FI6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FJ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FK6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FL6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="FM6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="FN6" s="34" t="inlineStr">
-        <is>
-          <t>feriado</t>
-        </is>
-      </c>
-      <c r="FO6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FP6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FQ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FR6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FS6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="FT6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="FU6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FV6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FW6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FX6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="FY6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="FZ6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="GA6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="GB6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GC6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="GD6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GE6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GF6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="GG6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="GH6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="GI6" s="34" t="inlineStr">
-        <is>
-          <t>feriado</t>
-        </is>
-      </c>
-      <c r="GJ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GK6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="GL6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GM6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GN6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="GO6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="GP6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GQ6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="GR6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GS6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="GT6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GU6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="GV6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="GW6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="GX6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GY6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="GZ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HA6" s="34" t="inlineStr">
-        <is>
-          <t>feriado</t>
-        </is>
-      </c>
-      <c r="HB6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="HC6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="HD6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HE6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HF6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HG6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HH6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HI6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="HJ6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="HK6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HL6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HM6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HN6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HO6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HP6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="HQ6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="HR6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HS6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HT6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="HU6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HV6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HW6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="HX6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="HY6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="HZ6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="IA6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="IB6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="IC6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="ID6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="IE6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="IF6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="IG6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="IH6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="II6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="IJ6" s="34" t="inlineStr">
-        <is>
-          <t>feriado</t>
-        </is>
-      </c>
-      <c r="IK6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="IL6" s="28" t="inlineStr">
-        <is>
-          <t>fds</t>
-        </is>
-      </c>
-      <c r="IM6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="IN6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="IO6" s="31" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="IP6" s="32" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-    </row>
+    <row r="6" ht="15.75" customHeight="1" thickBot="1"/>
     <row r="7" ht="15.75" customHeight="1" thickTop="1"/>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>

</xml_diff>